<commit_message>
schematics and netlist  added
</commit_message>
<xml_diff>
--- a/hardware/schematics/HUB-AUDIO-BOM.xlsx
+++ b/hardware/schematics/HUB-AUDIO-BOM.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="974" uniqueCount="531">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="974" uniqueCount="530">
   <si>
     <t>No.</t>
   </si>
@@ -55,13 +55,40 @@
     <t>1</t>
   </si>
   <si>
+    <t>1uF</t>
+  </si>
+  <si>
+    <t>C1,C24,C29,C35,C37,C39</t>
+  </si>
+  <si>
+    <t>C0402</t>
+  </si>
+  <si>
+    <t>Basic Part,Extended Part</t>
+  </si>
+  <si>
+    <t>1uF ±10% 25V,1uF ±10% 50V</t>
+  </si>
+  <si>
+    <t>CL05A105KA5NQNC,HGC0402R5105K500NTEJ</t>
+  </si>
+  <si>
+    <t>Capacitors:Multilayer Ceramic Capacitors MLCC - SMD/SMT</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>https://item.szlcsc.com/datasheet/CL05A105KA5NQNC/53938.html,https://item.szlcsc.com/datasheet/HGC0402R5105K500NTEJ/8532795.html</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
     <t>100nF</t>
   </si>
   <si>
-    <t>C1,C3,C4,C6,C8,C12,C102</t>
-  </si>
-  <si>
-    <t>C0402</t>
+    <t>C2,C3,C5,C22,C23,C109</t>
   </si>
   <si>
     <t>Basic Part</t>
@@ -73,64 +100,52 @@
     <t>CL05B104KB54PNC</t>
   </si>
   <si>
-    <t>Capacitors:Multilayer Ceramic Capacitors MLCC - SMD/SMT</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
     <t>https://item.szlcsc.com/datasheet/CL05B104KB54PNC/291005.html</t>
   </si>
   <si>
-    <t>2</t>
+    <t>3</t>
   </si>
   <si>
     <t>22uF</t>
   </si>
   <si>
-    <t>C2,C9,C13</t>
+    <t>C4,C9,C10</t>
   </si>
   <si>
     <t>C0805</t>
   </si>
   <si>
-    <t>22uF ±20% 25V</t>
-  </si>
-  <si>
-    <t>CL21A226MAQNNNE</t>
-  </si>
-  <si>
-    <t>https://item.szlcsc.com/datasheet/CL21A226MAQNNNE/46786.html</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>1uF</t>
-  </si>
-  <si>
-    <t>C5,C11,C14,C15,C16,C17,C19,C24,C30,C32,C34</t>
-  </si>
-  <si>
-    <t>Basic Part,Extended Part</t>
-  </si>
-  <si>
-    <t>1uF ±10% 25V,1uF ±10% 50V</t>
-  </si>
-  <si>
-    <t>CL05A105KA5NQNC,HGC0402R5105K500NTEJ</t>
-  </si>
-  <si>
-    <t>https://item.szlcsc.com/datasheet/CL05A105KA5NQNC/53938.html,https://item.szlcsc.com/datasheet/HGC0402R5105K500NTEJ/8532795.html</t>
+    <t>22uF ±20% 10V,22uF ±20% 25V</t>
+  </si>
+  <si>
+    <t>CL21A226MAQNNNE,CL21A226MPQNNNE</t>
+  </si>
+  <si>
+    <t>https://item.szlcsc.com/datasheet/CL21A226MAQNNNE/46786.html,https://item.szlcsc.com/datasheet/CL21A226MPQNNNE/30029.html</t>
   </si>
   <si>
     <t>4</t>
   </si>
   <si>
+    <t>C6,C8,C13,C14,C19,C20,C41,C50,C56,C57,C61,C63,C66,C69,C72,C73,C76,C77,C79,C80,C83,C89,C95,C101,C107,C110,C115,C120,C121,C124,C125,C132,C133,C136,C138,C141,C143,C145,C147,C153,C159,C165</t>
+  </si>
+  <si>
+    <t>Extended Part</t>
+  </si>
+  <si>
+    <t>0805X7R104K500NT,TCC0805X7R104K500DT</t>
+  </si>
+  <si>
+    <t>https://item.szlcsc.com/datasheet/0805X7R104K500NT/50843341.html,https://item.szlcsc.com/datasheet/TCC0805X7R104K500DT/268703.html</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
     <t>10uF</t>
   </si>
   <si>
-    <t>C7,C10,C18,C46,C47,C52,C53,C85,C86,C91,C92,C97,C98,C101,C109,C110,C115,C116,C121,C122,C127,C128,C133,C134,C139,C140</t>
+    <t>C7,C11,C21,C47,C48,C53,C54,C86,C87,C92,C93,C98,C99,C104,C105,C108,C117,C118,C129,C130,C139,C150,C151,C156,C157,C162,C163</t>
   </si>
   <si>
     <t>10uF ±10% 25V,10uF ±10% 50V</t>
@@ -145,16 +160,28 @@
     <t>CL21A106KAYNNNE_C15850,GRM21BR61H106KE43L</t>
   </si>
   <si>
-    <t>5</t>
+    <t>6</t>
+  </si>
+  <si>
+    <t>C12,C15,C16,C17,C18,C45,C49,C51,C55,C84,C88,C90,C94,C96,C100,C102,C106,C113,C119,C127,C131,C137,C140,C142,C144,C146,C148,C152,C154,C158,C160,C164</t>
+  </si>
+  <si>
+    <t>1uF ±10% 50V</t>
+  </si>
+  <si>
+    <t>CL21B105KBFNNNE</t>
+  </si>
+  <si>
+    <t>https://item.szlcsc.com/datasheet/CL21B105KBFNNNE/29074.html</t>
+  </si>
+  <si>
+    <t>7</t>
   </si>
   <si>
     <t>470nF</t>
   </si>
   <si>
-    <t>C20</t>
-  </si>
-  <si>
-    <t>Extended Part</t>
+    <t>C25</t>
   </si>
   <si>
     <t>470nF ±20% 50V</t>
@@ -166,13 +193,13 @@
     <t>https://item.szlcsc.com/datasheet/TCC0805X7R474M500FT/6236335.html</t>
   </si>
   <si>
-    <t>6</t>
+    <t>8</t>
   </si>
   <si>
     <t>8.2pF</t>
   </si>
   <si>
-    <t>C21,C22,C28</t>
+    <t>C26,C27,C33</t>
   </si>
   <si>
     <t>8.2pF 50V</t>
@@ -184,13 +211,13 @@
     <t>https://item.szlcsc.com/datasheet/CSA0402C0G8R2B500GT/50922894.html</t>
   </si>
   <si>
-    <t>7</t>
+    <t>9</t>
   </si>
   <si>
     <t>2.2nF</t>
   </si>
   <si>
-    <t>C23,C29,C31</t>
+    <t>C28,C34,C36</t>
   </si>
   <si>
     <t>2.2nF ±10% 25V</t>
@@ -202,10 +229,10 @@
     <t>https://atta.szlcsc.com/upload/public/pdf/source/20200615/C541386_7B176CE5F84559F9CFB8AA143269F5F2.pdf</t>
   </si>
   <si>
-    <t>8</t>
-  </si>
-  <si>
-    <t>C25</t>
+    <t>10</t>
+  </si>
+  <si>
+    <t>C30</t>
   </si>
   <si>
     <t>C0603</t>
@@ -220,10 +247,10 @@
     <t>https://item.szlcsc.com/datasheet/CC0603CPNPO9BN8R2/4415749.html</t>
   </si>
   <si>
-    <t>9</t>
-  </si>
-  <si>
-    <t>C26</t>
+    <t>11</t>
+  </si>
+  <si>
+    <t>C31</t>
   </si>
   <si>
     <t>2.2nF ±10% 50V</t>
@@ -235,13 +262,10 @@
     <t>https://item.szlcsc.com/datasheet/0603B222K500NT/1956.html</t>
   </si>
   <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t>C27</t>
-  </si>
-  <si>
-    <t>1uF ±10% 50V</t>
+    <t>12</t>
+  </si>
+  <si>
+    <t>C32</t>
   </si>
   <si>
     <t>CL10A105KB8NNNC</t>
@@ -250,13 +274,13 @@
     <t>https://item.szlcsc.com/datasheet/CL10A105KB8NNNC/16531.html</t>
   </si>
   <si>
-    <t>11</t>
+    <t>13</t>
   </si>
   <si>
     <t>15pF</t>
   </si>
   <si>
-    <t>C33,C35</t>
+    <t>C38,C40</t>
   </si>
   <si>
     <t>15pF ±5% 50V</t>
@@ -268,25 +292,13 @@
     <t>https://item.szlcsc.com/datasheet/0402CG150J500NT/1900.html</t>
   </si>
   <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>C36,C41,C43,C49,C55,C56,C60,C62,C65,C68,C71,C72,C75,C76,C78,C79,C82,C88,C94,C100,C103,C104,C105,C112,C118,C124,C130,C136,C142,C144,C149</t>
-  </si>
-  <si>
-    <t>0805X7R104K500NT,TCC0805X7R104K500DT</t>
-  </si>
-  <si>
-    <t>https://item.szlcsc.com/datasheet/0805X7R104K500NT/50843341.html,https://item.szlcsc.com/datasheet/TCC0805X7R104K500DT/268703.html</t>
-  </si>
-  <si>
-    <t>13</t>
+    <t>14</t>
   </si>
   <si>
     <t>33pF</t>
   </si>
   <si>
-    <t>C37</t>
+    <t>C42</t>
   </si>
   <si>
     <t>33pF ±5% 50V</t>
@@ -298,13 +310,13 @@
     <t>https://item.szlcsc.com/datasheet/CL05C330JB5NNNC/71562.html</t>
   </si>
   <si>
-    <t>14</t>
+    <t>15</t>
   </si>
   <si>
     <t>2.7pF</t>
   </si>
   <si>
-    <t>C38</t>
+    <t>C43</t>
   </si>
   <si>
     <t>±0.1pF 2.7pF 50V</t>
@@ -316,13 +328,13 @@
     <t>https://item.szlcsc.com/datasheet/GJM1555C1H2R7BB01D/78031.html</t>
   </si>
   <si>
-    <t>15</t>
+    <t>16</t>
   </si>
   <si>
     <t>18pF</t>
   </si>
   <si>
-    <t>C39</t>
+    <t>C44</t>
   </si>
   <si>
     <t>18pF ±5% 50V</t>
@@ -334,13 +346,133 @@
     <t>https://item.szlcsc.com/datasheet/0805CG180J500NT/2149.html</t>
   </si>
   <si>
-    <t>16</t>
+    <t>17</t>
+  </si>
+  <si>
+    <t>1nF</t>
+  </si>
+  <si>
+    <t>C46,C52,C85,C91,C97,C103,C116,C128,C149,C155,C161</t>
+  </si>
+  <si>
+    <t>1nF ±10% 50V</t>
+  </si>
+  <si>
+    <t>CC0805KRX7R9BB102</t>
+  </si>
+  <si>
+    <t>https://item.szlcsc.com/datasheet/CC0805KRX7R9BB102/95319.html</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>10nF</t>
+  </si>
+  <si>
+    <t>C58,C59,C64,C67,C70,C71,C74,C75,C78,C81,C82</t>
+  </si>
+  <si>
+    <t>10nF ±10% 50V</t>
+  </si>
+  <si>
+    <t>TCC0805X7R103K500DT</t>
+  </si>
+  <si>
+    <t>https://item.szlcsc.com/datasheet/TCC0805X7R103K500DT/268699.html</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>5.6nF</t>
+  </si>
+  <si>
+    <t>C60</t>
+  </si>
+  <si>
+    <t>5.6nF ±5% 50V</t>
+  </si>
+  <si>
+    <t>GRM2195C1H562JA01D</t>
+  </si>
+  <si>
+    <t>https://item.szlcsc.com/datasheet/GRM2195C1H562JA01D/78194.html</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>150pF</t>
+  </si>
+  <si>
+    <t>C62</t>
+  </si>
+  <si>
+    <t>150pF ±5% 50V</t>
+  </si>
+  <si>
+    <t>CC0805JRNPO9BN151</t>
+  </si>
+  <si>
+    <t>https://item.szlcsc.com/datasheet/CC0805JRNPO9BN151/108327.html</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>22pF</t>
+  </si>
+  <si>
+    <t>C65,C68,C112,C123</t>
+  </si>
+  <si>
+    <t>22pF ±1% 50V,22pF ±5% 50V</t>
+  </si>
+  <si>
+    <t>0805CG220F500NT,CL21C220JBANNNC</t>
+  </si>
+  <si>
+    <t>https://item.szlcsc.com/datasheet/0805CG220F500NT/208470.html,https://item.szlcsc.com/datasheet/CL21C220JBANNNC/2156.html</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>C111,C122</t>
+  </si>
+  <si>
+    <t>CC0805JRNPO9BN330</t>
+  </si>
+  <si>
+    <t>https://item.szlcsc.com/datasheet/CC0805JRNPO9BN330/108331.html</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>4.7uF</t>
+  </si>
+  <si>
+    <t>C114,C126</t>
+  </si>
+  <si>
+    <t>4.7uF ±10% 25V</t>
+  </si>
+  <si>
+    <t>CL21A475KAQNNNE</t>
+  </si>
+  <si>
+    <t>https://item.szlcsc.com/datasheet/CL21A475KAQNNNE/2131.html</t>
+  </si>
+  <si>
+    <t>24</t>
   </si>
   <si>
     <t>0.47pF</t>
   </si>
   <si>
-    <t>C40,C42</t>
+    <t>C134,C135</t>
   </si>
   <si>
     <t>0.47pF 50V ±0.25pF</t>
@@ -352,138 +484,6 @@
     <t>https://atta.szlcsc.com/upload/public/pdf/source/20200423/C519378_A803D508FCA1C9E05222E3A32899E571.pdf</t>
   </si>
   <si>
-    <t>17</t>
-  </si>
-  <si>
-    <t>C44,C48,C50,C54,C83,C87,C89,C93,C95,C99,C107,C111,C113,C117,C119,C123,C125,C129,C131,C135,C137,C141</t>
-  </si>
-  <si>
-    <t>CL21B105KBFNNNE</t>
-  </si>
-  <si>
-    <t>https://item.szlcsc.com/datasheet/CL21B105KBFNNNE/29074.html</t>
-  </si>
-  <si>
-    <t>18</t>
-  </si>
-  <si>
-    <t>1nF</t>
-  </si>
-  <si>
-    <t>C45,C51,C84,C90,C96,C108,C114,C120,C126,C132,C138</t>
-  </si>
-  <si>
-    <t>1nF ±10% 50V</t>
-  </si>
-  <si>
-    <t>CC0805KRX7R9BB102</t>
-  </si>
-  <si>
-    <t>https://item.szlcsc.com/datasheet/CC0805KRX7R9BB102/95319.html</t>
-  </si>
-  <si>
-    <t>19</t>
-  </si>
-  <si>
-    <t>10nF</t>
-  </si>
-  <si>
-    <t>C57,C59,C63,C66,C69,C70,C73,C74,C77,C80,C81</t>
-  </si>
-  <si>
-    <t>10nF ±10% 50V</t>
-  </si>
-  <si>
-    <t>TCC0805X7R103K500DT</t>
-  </si>
-  <si>
-    <t>https://item.szlcsc.com/datasheet/TCC0805X7R103K500DT/268699.html</t>
-  </si>
-  <si>
-    <t>20</t>
-  </si>
-  <si>
-    <t>5.6nF</t>
-  </si>
-  <si>
-    <t>C58</t>
-  </si>
-  <si>
-    <t>5.6nF ±5% 50V</t>
-  </si>
-  <si>
-    <t>GRM2195C1H562JA01D</t>
-  </si>
-  <si>
-    <t>https://item.szlcsc.com/datasheet/GRM2195C1H562JA01D/78194.html</t>
-  </si>
-  <si>
-    <t>21</t>
-  </si>
-  <si>
-    <t>150pF</t>
-  </si>
-  <si>
-    <t>C61</t>
-  </si>
-  <si>
-    <t>150pF ±5% 50V</t>
-  </si>
-  <si>
-    <t>CC0805JRNPO9BN151</t>
-  </si>
-  <si>
-    <t>https://item.szlcsc.com/datasheet/CC0805JRNPO9BN151/108327.html</t>
-  </si>
-  <si>
-    <t>22</t>
-  </si>
-  <si>
-    <t>22pF</t>
-  </si>
-  <si>
-    <t>C64,C67,C143,C147</t>
-  </si>
-  <si>
-    <t>22pF ±1% 50V,22pF ±5% 50V</t>
-  </si>
-  <si>
-    <t>0805CG220F500NT,CL21C220JBANNNC</t>
-  </si>
-  <si>
-    <t>https://item.szlcsc.com/datasheet/0805CG220F500NT/208470.html,https://item.szlcsc.com/datasheet/CL21C220JBANNNC/2156.html</t>
-  </si>
-  <si>
-    <t>23</t>
-  </si>
-  <si>
-    <t>4.7uF</t>
-  </si>
-  <si>
-    <t>C106,C145</t>
-  </si>
-  <si>
-    <t>4.7uF ±10% 25V</t>
-  </si>
-  <si>
-    <t>CL21A475KAQNNNE</t>
-  </si>
-  <si>
-    <t>https://item.szlcsc.com/datasheet/CL21A475KAQNNNE/2131.html</t>
-  </si>
-  <si>
-    <t>24</t>
-  </si>
-  <si>
-    <t>C146,C148</t>
-  </si>
-  <si>
-    <t>CC0805JRNPO9BN330</t>
-  </si>
-  <si>
-    <t>https://item.szlcsc.com/datasheet/CC0805JRNPO9BN330/108331.html</t>
-  </si>
-  <si>
     <t>25</t>
   </si>
   <si>
@@ -511,7 +511,7 @@
     <t>PJ-342</t>
   </si>
   <si>
-    <t>CN2,LINE_IN,LINE_OUT</t>
+    <t>CN2,LINE_IN1,LINE_OUT1</t>
   </si>
   <si>
     <t>AUDIO-SMD_PJ-342_C668606</t>
@@ -685,7 +685,7 @@
     <t>BLM21PG121SN1D</t>
   </si>
   <si>
-    <t>L1,L7,L8,L9,L10,L11,L13,L14,L15,L16,L17,L18</t>
+    <t>L1,L7,L8,L9,L10,L11,L12,L13,L15,L16,L17,L18</t>
   </si>
   <si>
     <t>L0805</t>
@@ -724,10 +724,34 @@
     <t>36</t>
   </si>
   <si>
+    <t>120nH</t>
+  </si>
+  <si>
+    <t>L3</t>
+  </si>
+  <si>
+    <t>L0402</t>
+  </si>
+  <si>
+    <t>120nH ±5%</t>
+  </si>
+  <si>
+    <t>LQW15ANR12J00D</t>
+  </si>
+  <si>
+    <t>Inductors, Coils, Chokes:Power Inductors</t>
+  </si>
+  <si>
+    <t>https://item.szlcsc.com/datasheet/LQW15ANR12J00D/114358.html</t>
+  </si>
+  <si>
+    <t>37</t>
+  </si>
+  <si>
     <t>22nH</t>
   </si>
   <si>
-    <t>L3</t>
+    <t>L4</t>
   </si>
   <si>
     <t>IND-SMD_L1.0-W0.5-2</t>
@@ -739,33 +763,9 @@
     <t>LQW15AN22NH00D</t>
   </si>
   <si>
-    <t>Inductors, Coils, Chokes:Power Inductors</t>
-  </si>
-  <si>
     <t>https://item.szlcsc.com/datasheet/LQW15AN22NH00D/738551.html</t>
   </si>
   <si>
-    <t>37</t>
-  </si>
-  <si>
-    <t>120nH</t>
-  </si>
-  <si>
-    <t>L4</t>
-  </si>
-  <si>
-    <t>L0402</t>
-  </si>
-  <si>
-    <t>120nH ±5%</t>
-  </si>
-  <si>
-    <t>LQW15ANR12J00D</t>
-  </si>
-  <si>
-    <t>https://item.szlcsc.com/datasheet/LQW15ANR12J00D/114358.html</t>
-  </si>
-  <si>
     <t>38</t>
   </si>
   <si>
@@ -808,7 +808,7 @@
     <t>LSQNB160808T470M</t>
   </si>
   <si>
-    <t>L12</t>
+    <t>L14</t>
   </si>
   <si>
     <t>适用于通用电子设备的绕线铁氧体功率电感器</t>
@@ -841,13 +841,34 @@
     <t>42</t>
   </si>
   <si>
+    <t>10kΩ</t>
+  </si>
+  <si>
+    <t>R1,R6,R7,R8,R31</t>
+  </si>
+  <si>
+    <t>R0402</t>
+  </si>
+  <si>
+    <t>10kΩ ±1% 62.5mW 厚膜电阻</t>
+  </si>
+  <si>
+    <t>0402WGF1002TCE</t>
+  </si>
+  <si>
+    <t>Resistors:Chip Resistor - Surface Mount</t>
+  </si>
+  <si>
+    <t>https://item.szlcsc.com/datasheet/0402WGF1002TCE/26487.html</t>
+  </si>
+  <si>
+    <t>43</t>
+  </si>
+  <si>
     <t>2kΩ</t>
   </si>
   <si>
-    <t>R1,R2</t>
-  </si>
-  <si>
-    <t>R0402</t>
+    <t>R2,R3</t>
   </si>
   <si>
     <t>2kΩ ±1% 62.5mW 厚膜电阻</t>
@@ -856,19 +877,16 @@
     <t>0402WGF2001TCE</t>
   </si>
   <si>
-    <t>Resistors:Chip Resistor - Surface Mount</t>
-  </si>
-  <si>
     <t>https://atta.szlcsc.com/upload/public/pdf/source/20200306/C422600_1E6D84923E4A46A82E41ADD87F860B5C.pdf</t>
   </si>
   <si>
-    <t>43</t>
+    <t>44</t>
   </si>
   <si>
     <t>5.1kΩ</t>
   </si>
   <si>
-    <t>R3,R4</t>
+    <t>R4,R5</t>
   </si>
   <si>
     <t>5.1kΩ ±1% 62.5mW 厚膜电阻</t>
@@ -880,31 +898,13 @@
     <t>https://item.szlcsc.com/datasheet/0402WGF5101TCE/26648.html</t>
   </si>
   <si>
-    <t>44</t>
-  </si>
-  <si>
-    <t>10kΩ</t>
-  </si>
-  <si>
-    <t>R5,R6,R31</t>
-  </si>
-  <si>
-    <t>10kΩ ±1% 62.5mW 厚膜电阻</t>
-  </si>
-  <si>
-    <t>0402WGF1002TCE</t>
-  </si>
-  <si>
-    <t>https://item.szlcsc.com/datasheet/0402WGF1002TCE/26487.html</t>
-  </si>
-  <si>
     <t>45</t>
   </si>
   <si>
     <t>100mΩ</t>
   </si>
   <si>
-    <t>R7,R8</t>
+    <t>R9,R10</t>
   </si>
   <si>
     <t>R2512</t>
@@ -928,7 +928,7 @@
     <t>1kΩ</t>
   </si>
   <si>
-    <t>R9,R13</t>
+    <t>R11,R15</t>
   </si>
   <si>
     <t>R0805</t>
@@ -943,7 +943,7 @@
     <t>47</t>
   </si>
   <si>
-    <t>R10,R11,R12,R14,R16,R17,R18,R19,R20,R21,R22,R23,R26,R27,R28,R29,R30,R33,R34</t>
+    <t>R12,R13,R14,R16,R18,R19,R20,R21,R22,R23,R24,R26,R27,R28,R29,R30,R32,R34,R35</t>
   </si>
   <si>
     <t>10kΩ ±1% 125mW 厚膜电阻,10kΩ ±5% 125mW 厚膜电阻</t>
@@ -961,7 +961,7 @@
     <t>10mΩ</t>
   </si>
   <si>
-    <t>R15</t>
+    <t>R17</t>
   </si>
   <si>
     <t>R1206</t>
@@ -1003,7 +1003,7 @@
     <t>56Ω</t>
   </si>
   <si>
-    <t>R32</t>
+    <t>R33</t>
   </si>
   <si>
     <t>56Ω ±1% 125mW 厚膜电阻</t>
@@ -1045,7 +1045,7 @@
     <t>33Ω</t>
   </si>
   <si>
-    <t>RN1,RN2,RN3,RN5</t>
+    <t>RN1,RN2,RN3,RN4</t>
   </si>
   <si>
     <t>RES-ARRAY-SMD_0603-4P-L1.6-W1.6-BL</t>
@@ -1066,7 +1066,7 @@
     <t>53</t>
   </si>
   <si>
-    <t>RN4</t>
+    <t>RN5</t>
   </si>
   <si>
     <t>RES-ARRAY-SMD_0603-8P-L3.2-W1.6-BL</t>
@@ -1102,10 +1102,34 @@
     <t>55</t>
   </si>
   <si>
+    <t>2.4GHz</t>
+  </si>
+  <si>
+    <t>U1</t>
+  </si>
+  <si>
+    <t>WIRELM-SMD_ESP32-S3-WROOM-1</t>
+  </si>
+  <si>
+    <t>不带固件 通用型Wi-Fi+低功耗蓝牙MCU模组</t>
+  </si>
+  <si>
+    <t>ESP32-S3-WROOM-1-N16</t>
+  </si>
+  <si>
+    <t>IoT/Communication Modules:WiFi Modules</t>
+  </si>
+  <si>
+    <t>https://item.szlcsc.com/datasheet/ESP32-S3-WROOM-1-N16/3198297.html</t>
+  </si>
+  <si>
+    <t>56</t>
+  </si>
+  <si>
     <t>24AA025E48T-I/OT</t>
   </si>
   <si>
-    <t>U1</t>
+    <t>U2</t>
   </si>
   <si>
     <t>带EUI-48或EUI-64节点标识的2K I2C串行EEPROM</t>
@@ -1117,30 +1141,6 @@
     <t>https://item.szlcsc.com/datasheet/24AA025E48T-I%252FOT/141182.html</t>
   </si>
   <si>
-    <t>56</t>
-  </si>
-  <si>
-    <t>2.4GHz</t>
-  </si>
-  <si>
-    <t>U2</t>
-  </si>
-  <si>
-    <t>WIRELM-SMD_ESP32-S3-WROOM-1</t>
-  </si>
-  <si>
-    <t>不带固件 通用型Wi-Fi+低功耗蓝牙MCU模组</t>
-  </si>
-  <si>
-    <t>ESP32-S3-WROOM-1-N16</t>
-  </si>
-  <si>
-    <t>IoT/Communication Modules:WiFi Modules</t>
-  </si>
-  <si>
-    <t>https://item.szlcsc.com/datasheet/ESP32-S3-WROOM-1-N16/3198297.html</t>
-  </si>
-  <si>
     <t>57</t>
   </si>
   <si>
@@ -1186,10 +1186,31 @@
     <t>59</t>
   </si>
   <si>
+    <t>TCA9555RTWR</t>
+  </si>
+  <si>
+    <t>U5,U21</t>
+  </si>
+  <si>
+    <t>VFQFPN-24_L4.0-W4.0-P0.50-BL-EP2.8</t>
+  </si>
+  <si>
+    <t>TCA9555 低电压16位 I²C 和 SMBus I/O 扩展器，带中断输出和配置寄存器</t>
+  </si>
+  <si>
+    <t>Interface:I/O Expanders</t>
+  </si>
+  <si>
+    <t>https://www.ti.com/cn/lit/gpn/tca9555</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
     <t>TPS7A2018PDQNR</t>
   </si>
   <si>
-    <t>U5</t>
+    <t>U6</t>
   </si>
   <si>
     <t>X2SON-4_L1.0-W1.0-P0.65-TL-EP</t>
@@ -1204,27 +1225,6 @@
     <t>https://www.ti.com/cn/lit/ds/symlink/tps7a20.pdf</t>
   </si>
   <si>
-    <t>60</t>
-  </si>
-  <si>
-    <t>TCA9555RTWR</t>
-  </si>
-  <si>
-    <t>U6,U21</t>
-  </si>
-  <si>
-    <t>VFQFPN-24_L4.0-W4.0-P0.50-BL-EP2.8</t>
-  </si>
-  <si>
-    <t>TCA9555 低电压16位 I²C 和 SMBus I/O 扩展器，带中断输出和配置寄存器</t>
-  </si>
-  <si>
-    <t>Interface:I/O Expanders</t>
-  </si>
-  <si>
-    <t>https://www.ti.com/cn/lit/gpn/tca9555</t>
-  </si>
-  <si>
     <t>61</t>
   </si>
   <si>
@@ -1450,16 +1450,34 @@
     <t>FSC-BT806</t>
   </si>
   <si>
-    <t>9369600</t>
-  </si>
-  <si>
     <t>73</t>
   </si>
   <si>
+    <t>SC16IS740IPW,128</t>
+  </si>
+  <si>
+    <t>U23,U25</t>
+  </si>
+  <si>
+    <t>TSSOP-16_L5.0-W4.4-P0.65-LS6.4-BL</t>
+  </si>
+  <si>
+    <t>单路通用异步收发传输器（UART），具备I2C总线/SPI接口，64字节收发FIFO，内置IrDA SIR支持</t>
+  </si>
+  <si>
+    <t>Interface:UART</t>
+  </si>
+  <si>
+    <t>https://www.nxp.com.cn/docs/en/data-sheet/SC16IS740_750_760.pdf</t>
+  </si>
+  <si>
+    <t>74</t>
+  </si>
+  <si>
     <t>FSC-BT1026x</t>
   </si>
   <si>
-    <t>U23</t>
+    <t>U24</t>
   </si>
   <si>
     <t>Bluetooth:FSC-BT1026x</t>
@@ -1468,13 +1486,13 @@
     <t>Bluetooth:</t>
   </si>
   <si>
-    <t>74</t>
+    <t>75</t>
   </si>
   <si>
     <t>SN75451BDR</t>
   </si>
   <si>
-    <t>U24</t>
+    <t>U26</t>
   </si>
   <si>
     <t>SOIC-8_L5.0-W4.0-P1.27-LS6.0-BL</t>
@@ -1489,13 +1507,13 @@
     <t>https://www.ti.com/cn/lit/gpn/sn75453b</t>
   </si>
   <si>
-    <t>75</t>
+    <t>76</t>
   </si>
   <si>
     <t>HFBR-1521Z</t>
   </si>
   <si>
-    <t>U25</t>
+    <t>U27</t>
   </si>
   <si>
     <t>CONN-TH_HFBR-1521Z</t>
@@ -1504,13 +1522,13 @@
     <t>https://item.szlcsc.com/datasheet/HFBR-1521Z/200120.html</t>
   </si>
   <si>
-    <t>76</t>
+    <t>77</t>
   </si>
   <si>
     <t>TLV320AIC3104IRHBR</t>
   </si>
   <si>
-    <t>U26</t>
+    <t>U28</t>
   </si>
   <si>
     <t>HVQFN-32_L5.0-W5.0-P0.50-TL-EP</t>
@@ -1523,27 +1541,6 @@
   </si>
   <si>
     <t>https://www.ti.com/cn/lit/gpn/tlv320aic3104</t>
-  </si>
-  <si>
-    <t>77</t>
-  </si>
-  <si>
-    <t>SC16IS740IPW,128</t>
-  </si>
-  <si>
-    <t>U27,U28</t>
-  </si>
-  <si>
-    <t>TSSOP-16_L5.0-W4.4-P0.65-LS6.4-BL</t>
-  </si>
-  <si>
-    <t>单路通用异步收发传输器（UART），具备I2C总线/SPI接口，64字节收发FIFO，内置IrDA SIR支持</t>
-  </si>
-  <si>
-    <t>Interface:UART</t>
-  </si>
-  <si>
-    <t>https://www.nxp.com.cn/docs/en/data-sheet/SC16IS740_750_760.pdf</t>
   </si>
   <si>
     <t>78</t>
@@ -2032,7 +2029,7 @@
         <v>13</v>
       </c>
       <c r="B2">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C2" t="s">
         <v>14</v>
@@ -2073,7 +2070,7 @@
         <v>23</v>
       </c>
       <c r="B3">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C3" t="s">
         <v>24</v>
@@ -2082,10 +2079,10 @@
         <v>25</v>
       </c>
       <c r="E3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" t="s">
         <v>26</v>
-      </c>
-      <c r="F3" t="s">
-        <v>17</v>
       </c>
       <c r="G3" t="s">
         <v>27</v>
@@ -2114,7 +2111,7 @@
         <v>30</v>
       </c>
       <c r="B4">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="C4" t="s">
         <v>31</v>
@@ -2123,10 +2120,10 @@
         <v>32</v>
       </c>
       <c r="E4" t="s">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="F4" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="G4" t="s">
         <v>34</v>
@@ -2155,25 +2152,25 @@
         <v>37</v>
       </c>
       <c r="B5">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="C5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" t="s">
         <v>38</v>
       </c>
-      <c r="D5" t="s">
-        <v>39</v>
-      </c>
       <c r="E5" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="F5" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="G5" t="s">
+        <v>27</v>
+      </c>
+      <c r="H5" t="s">
         <v>40</v>
-      </c>
-      <c r="H5" t="s">
-        <v>41</v>
       </c>
       <c r="I5" t="s">
         <v>20</v>
@@ -2182,39 +2179,39 @@
         <v>21</v>
       </c>
       <c r="K5" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="L5" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="M5" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6">
+        <v>27</v>
+      </c>
+      <c r="C6" t="s">
+        <v>43</v>
+      </c>
+      <c r="D6" t="s">
         <v>44</v>
       </c>
-      <c r="B6">
-        <v>1</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="E6" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G6" t="s">
         <v>45</v>
       </c>
-      <c r="D6" t="s">
+      <c r="H6" t="s">
         <v>46</v>
-      </c>
-      <c r="E6" t="s">
-        <v>26</v>
-      </c>
-      <c r="F6" t="s">
-        <v>47</v>
-      </c>
-      <c r="G6" t="s">
-        <v>48</v>
-      </c>
-      <c r="H6" t="s">
-        <v>49</v>
       </c>
       <c r="I6" t="s">
         <v>20</v>
@@ -2223,39 +2220,39 @@
         <v>21</v>
       </c>
       <c r="K6" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="L6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="M6" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>49</v>
+      </c>
+      <c r="B7">
+        <v>32</v>
+      </c>
+      <c r="C7" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" t="s">
+        <v>50</v>
+      </c>
+      <c r="E7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G7" t="s">
         <v>51</v>
       </c>
-      <c r="B7">
-        <v>3</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="H7" t="s">
         <v>52</v>
-      </c>
-      <c r="D7" t="s">
-        <v>53</v>
-      </c>
-      <c r="E7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F7" t="s">
-        <v>47</v>
-      </c>
-      <c r="G7" t="s">
-        <v>54</v>
-      </c>
-      <c r="H7" t="s">
-        <v>55</v>
       </c>
       <c r="I7" t="s">
         <v>20</v>
@@ -2264,39 +2261,39 @@
         <v>21</v>
       </c>
       <c r="K7" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="L7" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="M7" t="s">
-        <v>52</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B8">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8" t="s">
+        <v>33</v>
+      </c>
+      <c r="F8" t="s">
+        <v>39</v>
+      </c>
+      <c r="G8" t="s">
         <v>57</v>
       </c>
-      <c r="B8">
-        <v>3</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="H8" t="s">
         <v>58</v>
-      </c>
-      <c r="D8" t="s">
-        <v>59</v>
-      </c>
-      <c r="E8" t="s">
-        <v>16</v>
-      </c>
-      <c r="F8" t="s">
-        <v>47</v>
-      </c>
-      <c r="G8" t="s">
-        <v>60</v>
-      </c>
-      <c r="H8" t="s">
-        <v>61</v>
       </c>
       <c r="I8" t="s">
         <v>20</v>
@@ -2305,39 +2302,39 @@
         <v>21</v>
       </c>
       <c r="K8" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="L8" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="M8" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>60</v>
+      </c>
+      <c r="B9">
+        <v>3</v>
+      </c>
+      <c r="C9" t="s">
+        <v>61</v>
+      </c>
+      <c r="D9" t="s">
+        <v>62</v>
+      </c>
+      <c r="E9" t="s">
+        <v>16</v>
+      </c>
+      <c r="F9" t="s">
+        <v>39</v>
+      </c>
+      <c r="G9" t="s">
         <v>63</v>
       </c>
-      <c r="B9">
-        <v>1</v>
-      </c>
-      <c r="C9" t="s">
-        <v>52</v>
-      </c>
-      <c r="D9" t="s">
+      <c r="H9" t="s">
         <v>64</v>
-      </c>
-      <c r="E9" t="s">
-        <v>65</v>
-      </c>
-      <c r="F9" t="s">
-        <v>47</v>
-      </c>
-      <c r="G9" t="s">
-        <v>66</v>
-      </c>
-      <c r="H9" t="s">
-        <v>67</v>
       </c>
       <c r="I9" t="s">
         <v>20</v>
@@ -2346,39 +2343,39 @@
         <v>21</v>
       </c>
       <c r="K9" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="L9" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="M9" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>66</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>67</v>
+      </c>
+      <c r="D10" t="s">
+        <v>68</v>
+      </c>
+      <c r="E10" t="s">
+        <v>16</v>
+      </c>
+      <c r="F10" t="s">
+        <v>39</v>
+      </c>
+      <c r="G10" t="s">
         <v>69</v>
       </c>
-      <c r="B10">
-        <v>1</v>
-      </c>
-      <c r="C10" t="s">
-        <v>58</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="H10" t="s">
         <v>70</v>
-      </c>
-      <c r="E10" t="s">
-        <v>65</v>
-      </c>
-      <c r="F10" t="s">
-        <v>17</v>
-      </c>
-      <c r="G10" t="s">
-        <v>71</v>
-      </c>
-      <c r="H10" t="s">
-        <v>72</v>
       </c>
       <c r="I10" t="s">
         <v>20</v>
@@ -2387,39 +2384,39 @@
         <v>21</v>
       </c>
       <c r="K10" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="L10" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="M10" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B11">
         <v>1</v>
       </c>
       <c r="C11" t="s">
-        <v>31</v>
+        <v>61</v>
       </c>
       <c r="D11" t="s">
+        <v>73</v>
+      </c>
+      <c r="E11" t="s">
+        <v>74</v>
+      </c>
+      <c r="F11" t="s">
+        <v>39</v>
+      </c>
+      <c r="G11" t="s">
         <v>75</v>
       </c>
-      <c r="E11" t="s">
-        <v>65</v>
-      </c>
-      <c r="F11" t="s">
-        <v>17</v>
-      </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>76</v>
-      </c>
-      <c r="H11" t="s">
-        <v>77</v>
       </c>
       <c r="I11" t="s">
         <v>20</v>
@@ -2428,39 +2425,39 @@
         <v>21</v>
       </c>
       <c r="K11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="L11" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="M11" t="s">
-        <v>31</v>
+        <v>61</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>78</v>
+      </c>
+      <c r="B12">
+        <v>1</v>
+      </c>
+      <c r="C12" t="s">
+        <v>67</v>
+      </c>
+      <c r="D12" t="s">
         <v>79</v>
       </c>
-      <c r="B12">
-        <v>2</v>
-      </c>
-      <c r="C12" t="s">
+      <c r="E12" t="s">
+        <v>74</v>
+      </c>
+      <c r="F12" t="s">
+        <v>26</v>
+      </c>
+      <c r="G12" t="s">
         <v>80</v>
       </c>
-      <c r="D12" t="s">
+      <c r="H12" t="s">
         <v>81</v>
-      </c>
-      <c r="E12" t="s">
-        <v>16</v>
-      </c>
-      <c r="F12" t="s">
-        <v>17</v>
-      </c>
-      <c r="G12" t="s">
-        <v>82</v>
-      </c>
-      <c r="H12" t="s">
-        <v>83</v>
       </c>
       <c r="I12" t="s">
         <v>20</v>
@@ -2469,39 +2466,39 @@
         <v>21</v>
       </c>
       <c r="K12" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="L12" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="M12" t="s">
-        <v>80</v>
+        <v>67</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B13">
-        <v>31</v>
+        <v>1</v>
       </c>
       <c r="C13" t="s">
         <v>14</v>
       </c>
       <c r="D13" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E13" t="s">
+        <v>74</v>
+      </c>
+      <c r="F13" t="s">
         <v>26</v>
       </c>
-      <c r="F13" t="s">
-        <v>47</v>
-      </c>
       <c r="G13" t="s">
-        <v>18</v>
+        <v>51</v>
       </c>
       <c r="H13" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="I13" t="s">
         <v>20</v>
@@ -2510,10 +2507,10 @@
         <v>21</v>
       </c>
       <c r="K13" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="L13" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="M13" t="s">
         <v>14</v>
@@ -2521,28 +2518,28 @@
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>87</v>
+      </c>
+      <c r="B14">
+        <v>2</v>
+      </c>
+      <c r="C14" t="s">
+        <v>88</v>
+      </c>
+      <c r="D14" t="s">
         <v>89</v>
-      </c>
-      <c r="B14">
-        <v>1</v>
-      </c>
-      <c r="C14" t="s">
-        <v>90</v>
-      </c>
-      <c r="D14" t="s">
-        <v>91</v>
       </c>
       <c r="E14" t="s">
         <v>16</v>
       </c>
       <c r="F14" t="s">
-        <v>47</v>
+        <v>26</v>
       </c>
       <c r="G14" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H14" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="I14" t="s">
         <v>20</v>
@@ -2551,39 +2548,39 @@
         <v>21</v>
       </c>
       <c r="K14" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="L14" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="M14" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B15">
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D15" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="E15" t="s">
         <v>16</v>
       </c>
       <c r="F15" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G15" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="H15" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="I15" t="s">
         <v>20</v>
@@ -2592,39 +2589,39 @@
         <v>21</v>
       </c>
       <c r="K15" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="L15" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="M15" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B16">
         <v>1</v>
       </c>
       <c r="C16" t="s">
+        <v>100</v>
+      </c>
+      <c r="D16" t="s">
+        <v>101</v>
+      </c>
+      <c r="E16" t="s">
+        <v>16</v>
+      </c>
+      <c r="F16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G16" t="s">
         <v>102</v>
       </c>
-      <c r="D16" t="s">
+      <c r="H16" t="s">
         <v>103</v>
-      </c>
-      <c r="E16" t="s">
-        <v>26</v>
-      </c>
-      <c r="F16" t="s">
-        <v>47</v>
-      </c>
-      <c r="G16" t="s">
-        <v>104</v>
-      </c>
-      <c r="H16" t="s">
-        <v>105</v>
       </c>
       <c r="I16" t="s">
         <v>20</v>
@@ -2633,39 +2630,39 @@
         <v>21</v>
       </c>
       <c r="K16" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="L16" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="M16" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>105</v>
+      </c>
+      <c r="B17">
+        <v>1</v>
+      </c>
+      <c r="C17" t="s">
+        <v>106</v>
+      </c>
+      <c r="D17" t="s">
         <v>107</v>
       </c>
-      <c r="B17">
-        <v>2</v>
-      </c>
-      <c r="C17" t="s">
+      <c r="E17" t="s">
+        <v>33</v>
+      </c>
+      <c r="F17" t="s">
+        <v>39</v>
+      </c>
+      <c r="G17" t="s">
         <v>108</v>
       </c>
-      <c r="D17" t="s">
+      <c r="H17" t="s">
         <v>109</v>
-      </c>
-      <c r="E17" t="s">
-        <v>65</v>
-      </c>
-      <c r="F17" t="s">
-        <v>47</v>
-      </c>
-      <c r="G17" t="s">
-        <v>110</v>
-      </c>
-      <c r="H17" t="s">
-        <v>111</v>
       </c>
       <c r="I17" t="s">
         <v>20</v>
@@ -2674,36 +2671,36 @@
         <v>21</v>
       </c>
       <c r="K17" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="L17" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="M17" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>111</v>
+      </c>
+      <c r="B18">
+        <v>11</v>
+      </c>
+      <c r="C18" t="s">
+        <v>112</v>
+      </c>
+      <c r="D18" t="s">
         <v>113</v>
       </c>
-      <c r="B18">
-        <v>22</v>
-      </c>
-      <c r="C18" t="s">
-        <v>31</v>
-      </c>
-      <c r="D18" t="s">
+      <c r="E18" t="s">
+        <v>33</v>
+      </c>
+      <c r="F18" t="s">
+        <v>39</v>
+      </c>
+      <c r="G18" t="s">
         <v>114</v>
-      </c>
-      <c r="E18" t="s">
-        <v>26</v>
-      </c>
-      <c r="F18" t="s">
-        <v>17</v>
-      </c>
-      <c r="G18" t="s">
-        <v>76</v>
       </c>
       <c r="H18" t="s">
         <v>115</v>
@@ -2721,7 +2718,7 @@
         <v>115</v>
       </c>
       <c r="M18" t="s">
-        <v>31</v>
+        <v>112</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.25">
@@ -2738,10 +2735,10 @@
         <v>119</v>
       </c>
       <c r="E19" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="F19" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G19" t="s">
         <v>120</v>
@@ -2770,7 +2767,7 @@
         <v>123</v>
       </c>
       <c r="B20">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="C20" t="s">
         <v>124</v>
@@ -2779,10 +2776,10 @@
         <v>125</v>
       </c>
       <c r="E20" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="F20" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G20" t="s">
         <v>126</v>
@@ -2820,10 +2817,10 @@
         <v>131</v>
       </c>
       <c r="E21" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="F21" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G21" t="s">
         <v>132</v>
@@ -2852,7 +2849,7 @@
         <v>135</v>
       </c>
       <c r="B22">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C22" t="s">
         <v>136</v>
@@ -2861,10 +2858,10 @@
         <v>137</v>
       </c>
       <c r="E22" t="s">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="F22" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="G22" t="s">
         <v>138</v>
@@ -2893,25 +2890,25 @@
         <v>141</v>
       </c>
       <c r="B23">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C23" t="s">
+        <v>94</v>
+      </c>
+      <c r="D23" t="s">
         <v>142</v>
       </c>
-      <c r="D23" t="s">
+      <c r="E23" t="s">
+        <v>33</v>
+      </c>
+      <c r="F23" t="s">
+        <v>39</v>
+      </c>
+      <c r="G23" t="s">
+        <v>96</v>
+      </c>
+      <c r="H23" t="s">
         <v>143</v>
-      </c>
-      <c r="E23" t="s">
-        <v>26</v>
-      </c>
-      <c r="F23" t="s">
-        <v>33</v>
-      </c>
-      <c r="G23" t="s">
-        <v>144</v>
-      </c>
-      <c r="H23" t="s">
-        <v>145</v>
       </c>
       <c r="I23" t="s">
         <v>20</v>
@@ -2920,39 +2917,39 @@
         <v>21</v>
       </c>
       <c r="K23" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="L23" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="M23" t="s">
-        <v>142</v>
+        <v>94</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B24">
         <v>2</v>
       </c>
       <c r="C24" t="s">
+        <v>146</v>
+      </c>
+      <c r="D24" t="s">
+        <v>147</v>
+      </c>
+      <c r="E24" t="s">
+        <v>33</v>
+      </c>
+      <c r="F24" t="s">
+        <v>26</v>
+      </c>
+      <c r="G24" t="s">
         <v>148</v>
       </c>
-      <c r="D24" t="s">
+      <c r="H24" t="s">
         <v>149</v>
-      </c>
-      <c r="E24" t="s">
-        <v>26</v>
-      </c>
-      <c r="F24" t="s">
-        <v>17</v>
-      </c>
-      <c r="G24" t="s">
-        <v>150</v>
-      </c>
-      <c r="H24" t="s">
-        <v>151</v>
       </c>
       <c r="I24" t="s">
         <v>20</v>
@@ -2961,36 +2958,36 @@
         <v>21</v>
       </c>
       <c r="K24" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="L24" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="M24" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B25">
         <v>2</v>
       </c>
       <c r="C25" t="s">
-        <v>90</v>
+        <v>152</v>
       </c>
       <c r="D25" t="s">
+        <v>153</v>
+      </c>
+      <c r="E25" t="s">
+        <v>74</v>
+      </c>
+      <c r="F25" t="s">
+        <v>39</v>
+      </c>
+      <c r="G25" t="s">
         <v>154</v>
-      </c>
-      <c r="E25" t="s">
-        <v>26</v>
-      </c>
-      <c r="F25" t="s">
-        <v>47</v>
-      </c>
-      <c r="G25" t="s">
-        <v>92</v>
       </c>
       <c r="H25" t="s">
         <v>155</v>
@@ -3008,7 +3005,7 @@
         <v>155</v>
       </c>
       <c r="M25" t="s">
-        <v>90</v>
+        <v>152</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.25">
@@ -3028,7 +3025,7 @@
         <v>160</v>
       </c>
       <c r="F26" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G26" t="s">
         <v>161</v>
@@ -3069,7 +3066,7 @@
         <v>167</v>
       </c>
       <c r="F27" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G27" t="s">
         <v>168</v>
@@ -3110,7 +3107,7 @@
         <v>175</v>
       </c>
       <c r="F28" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="G28" t="s">
         <v>176</v>
@@ -3151,7 +3148,7 @@
         <v>183</v>
       </c>
       <c r="F29" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G29" t="s">
         <v>184</v>
@@ -3192,7 +3189,7 @@
         <v>191</v>
       </c>
       <c r="F30" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="G30" t="s">
         <v>192</v>
@@ -3233,7 +3230,7 @@
         <v>198</v>
       </c>
       <c r="F31" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G31" t="s">
         <v>199</v>
@@ -3274,7 +3271,7 @@
         <v>204</v>
       </c>
       <c r="F32" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G32" t="s">
         <v>205</v>
@@ -3315,7 +3312,7 @@
         <v>211</v>
       </c>
       <c r="F33" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G33" t="s">
         <v>212</v>
@@ -3356,7 +3353,7 @@
         <v>218</v>
       </c>
       <c r="F34" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G34" t="s">
         <v>219</v>
@@ -3397,7 +3394,7 @@
         <v>225</v>
       </c>
       <c r="F35" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G35" t="s">
         <v>226</v>
@@ -3438,7 +3435,7 @@
         <v>231</v>
       </c>
       <c r="F36" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G36" t="s">
         <v>232</v>
@@ -3479,7 +3476,7 @@
         <v>239</v>
       </c>
       <c r="F37" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G37" t="s">
         <v>240</v>
@@ -3520,7 +3517,7 @@
         <v>247</v>
       </c>
       <c r="F38" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G38" t="s">
         <v>248</v>
@@ -3561,7 +3558,7 @@
         <v>204</v>
       </c>
       <c r="F39" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G39" t="s">
         <v>254</v>
@@ -3602,7 +3599,7 @@
         <v>204</v>
       </c>
       <c r="F40" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G40" t="s">
         <v>260</v>
@@ -3643,7 +3640,7 @@
         <v>204</v>
       </c>
       <c r="F41" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G41" t="s">
         <v>266</v>
@@ -3684,7 +3681,7 @@
         <v>271</v>
       </c>
       <c r="F42" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G42" t="s">
         <v>272</v>
@@ -3713,7 +3710,7 @@
         <v>275</v>
       </c>
       <c r="B43">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C43" t="s">
         <v>276</v>
@@ -3725,7 +3722,7 @@
         <v>278</v>
       </c>
       <c r="F43" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="G43" t="s">
         <v>279</v>
@@ -3766,7 +3763,7 @@
         <v>278</v>
       </c>
       <c r="F44" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="G44" t="s">
         <v>286</v>
@@ -3795,7 +3792,7 @@
         <v>289</v>
       </c>
       <c r="B45">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C45" t="s">
         <v>290</v>
@@ -3807,7 +3804,7 @@
         <v>278</v>
       </c>
       <c r="F45" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="G45" t="s">
         <v>292</v>
@@ -3848,7 +3845,7 @@
         <v>298</v>
       </c>
       <c r="F46" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G46" t="s">
         <v>299</v>
@@ -3889,7 +3886,7 @@
         <v>306</v>
       </c>
       <c r="F47" t="s">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="G47" t="s">
         <v>307</v>
@@ -3904,7 +3901,7 @@
         <v>21</v>
       </c>
       <c r="K47" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="L47" t="s">
         <v>308</v>
@@ -3921,7 +3918,7 @@
         <v>19</v>
       </c>
       <c r="C48" t="s">
-        <v>290</v>
+        <v>276</v>
       </c>
       <c r="D48" t="s">
         <v>310</v>
@@ -3930,7 +3927,7 @@
         <v>306</v>
       </c>
       <c r="F48" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="G48" t="s">
         <v>311</v>
@@ -3951,7 +3948,7 @@
         <v>312</v>
       </c>
       <c r="M48" t="s">
-        <v>290</v>
+        <v>276</v>
       </c>
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.25">
@@ -3971,7 +3968,7 @@
         <v>317</v>
       </c>
       <c r="F49" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G49" t="s">
         <v>318</v>
@@ -4012,7 +4009,7 @@
         <v>306</v>
       </c>
       <c r="F50" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G50" t="s">
         <v>325</v>
@@ -4053,7 +4050,7 @@
         <v>306</v>
       </c>
       <c r="F51" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G51" t="s">
         <v>331</v>
@@ -4094,7 +4091,7 @@
         <v>337</v>
       </c>
       <c r="F52" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G52" t="s">
         <v>338</v>
@@ -4135,7 +4132,7 @@
         <v>345</v>
       </c>
       <c r="F53" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G53" t="s">
         <v>346</v>
@@ -4176,7 +4173,7 @@
         <v>352</v>
       </c>
       <c r="F54" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G54" t="s">
         <v>346</v>
@@ -4217,7 +4214,7 @@
         <v>358</v>
       </c>
       <c r="F55" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G55" t="s">
         <v>359</v>
@@ -4255,28 +4252,28 @@
         <v>364</v>
       </c>
       <c r="E56" t="s">
-        <v>271</v>
+        <v>365</v>
       </c>
       <c r="F56" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G56" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="H56" t="s">
-        <v>363</v>
+        <v>367</v>
       </c>
       <c r="I56" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="J56" t="s">
         <v>21</v>
       </c>
       <c r="K56" t="s">
+        <v>369</v>
+      </c>
+      <c r="L56" t="s">
         <v>367</v>
-      </c>
-      <c r="L56" t="s">
-        <v>363</v>
       </c>
       <c r="M56" t="s">
         <v>363</v>
@@ -4284,28 +4281,28 @@
     </row>
     <row r="57" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B57">
         <v>1</v>
       </c>
       <c r="C57" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="D57" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="E57" t="s">
+        <v>271</v>
+      </c>
+      <c r="F57" t="s">
+        <v>39</v>
+      </c>
+      <c r="G57" t="s">
+        <v>373</v>
+      </c>
+      <c r="H57" t="s">
         <v>371</v>
-      </c>
-      <c r="F57" t="s">
-        <v>47</v>
-      </c>
-      <c r="G57" t="s">
-        <v>372</v>
-      </c>
-      <c r="H57" t="s">
-        <v>373</v>
       </c>
       <c r="I57" t="s">
         <v>374</v>
@@ -4317,10 +4314,10 @@
         <v>375</v>
       </c>
       <c r="L57" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="M57" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
     </row>
     <row r="58" spans="1:13" x14ac:dyDescent="0.25">
@@ -4340,7 +4337,7 @@
         <v>379</v>
       </c>
       <c r="F58" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G58" t="s">
         <v>380</v>
@@ -4381,7 +4378,7 @@
         <v>386</v>
       </c>
       <c r="F59" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G59" t="s">
         <v>387</v>
@@ -4410,7 +4407,7 @@
         <v>390</v>
       </c>
       <c r="B60">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C60" t="s">
         <v>391</v>
@@ -4422,7 +4419,7 @@
         <v>393</v>
       </c>
       <c r="F60" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G60" t="s">
         <v>394</v>
@@ -4451,7 +4448,7 @@
         <v>397</v>
       </c>
       <c r="B61">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C61" t="s">
         <v>398</v>
@@ -4463,7 +4460,7 @@
         <v>400</v>
       </c>
       <c r="F61" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G61" t="s">
         <v>401</v>
@@ -4501,10 +4498,10 @@
         <v>406</v>
       </c>
       <c r="E62" t="s">
-        <v>393</v>
+        <v>400</v>
       </c>
       <c r="F62" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G62" t="s">
         <v>405</v>
@@ -4513,7 +4510,7 @@
         <v>405</v>
       </c>
       <c r="I62" t="s">
-        <v>395</v>
+        <v>402</v>
       </c>
       <c r="J62" t="s">
         <v>21</v>
@@ -4545,7 +4542,7 @@
         <v>410</v>
       </c>
       <c r="F63" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G63" t="s">
         <v>411</v>
@@ -4586,7 +4583,7 @@
         <v>417</v>
       </c>
       <c r="F64" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G64" t="s">
         <v>418</v>
@@ -4627,7 +4624,7 @@
         <v>424</v>
       </c>
       <c r="F65" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G65" t="s">
         <v>425</v>
@@ -4668,7 +4665,7 @@
         <v>430</v>
       </c>
       <c r="F66" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G66" t="s">
         <v>431</v>
@@ -4709,7 +4706,7 @@
         <v>437</v>
       </c>
       <c r="F67" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G67" t="s">
         <v>438</v>
@@ -4750,7 +4747,7 @@
         <v>445</v>
       </c>
       <c r="F68" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G68" t="s">
         <v>446</v>
@@ -4791,7 +4788,7 @@
         <v>452</v>
       </c>
       <c r="F69" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G69" t="s">
         <v>453</v>
@@ -4832,7 +4829,7 @@
         <v>459</v>
       </c>
       <c r="F70" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G70" t="s">
         <v>460</v>
@@ -4873,7 +4870,7 @@
         <v>466</v>
       </c>
       <c r="F71" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G71" t="s">
         <v>464</v>
@@ -4914,7 +4911,7 @@
         <v>472</v>
       </c>
       <c r="F72" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G72" t="s">
         <v>473</v>
@@ -4923,7 +4920,7 @@
         <v>470</v>
       </c>
       <c r="I72" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="J72" t="s">
         <v>21</v>
@@ -4967,7 +4964,7 @@
         <v>21</v>
       </c>
       <c r="J73" t="s">
-        <v>479</v>
+        <v>172</v>
       </c>
       <c r="K73" t="s">
         <v>21</v>
@@ -4981,274 +4978,274 @@
     </row>
     <row r="74" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
+        <v>479</v>
+      </c>
+      <c r="B74">
+        <v>2</v>
+      </c>
+      <c r="C74" t="s">
         <v>480</v>
       </c>
-      <c r="B74">
-        <v>1</v>
-      </c>
-      <c r="C74" t="s">
+      <c r="D74" t="s">
         <v>481</v>
       </c>
-      <c r="D74" t="s">
+      <c r="E74" t="s">
         <v>482</v>
       </c>
-      <c r="E74" t="s">
+      <c r="F74" t="s">
+        <v>39</v>
+      </c>
+      <c r="G74" t="s">
         <v>483</v>
       </c>
-      <c r="F74" t="s">
-        <v>21</v>
-      </c>
-      <c r="G74" t="s">
-        <v>21</v>
-      </c>
       <c r="H74" t="s">
-        <v>21</v>
+        <v>480</v>
       </c>
       <c r="I74" t="s">
         <v>484</v>
       </c>
       <c r="J74" t="s">
-        <v>479</v>
+        <v>21</v>
       </c>
       <c r="K74" t="s">
-        <v>21</v>
+        <v>485</v>
       </c>
       <c r="L74" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="M74" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
     </row>
     <row r="75" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="B75">
         <v>1</v>
       </c>
       <c r="C75" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="D75" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="E75" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="F75" t="s">
-        <v>47</v>
+        <v>21</v>
       </c>
       <c r="G75" t="s">
-        <v>489</v>
+        <v>21</v>
       </c>
       <c r="H75" t="s">
-        <v>486</v>
+        <v>21</v>
       </c>
       <c r="I75" t="s">
         <v>490</v>
       </c>
       <c r="J75" t="s">
-        <v>21</v>
+        <v>172</v>
       </c>
       <c r="K75" t="s">
-        <v>491</v>
+        <v>21</v>
       </c>
       <c r="L75" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="M75" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
     </row>
     <row r="76" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="B76">
         <v>1</v>
       </c>
       <c r="C76" t="s">
+        <v>492</v>
+      </c>
+      <c r="D76" t="s">
         <v>493</v>
       </c>
-      <c r="D76" t="s">
+      <c r="E76" t="s">
         <v>494</v>
       </c>
-      <c r="E76" t="s">
+      <c r="F76" t="s">
+        <v>39</v>
+      </c>
+      <c r="G76" t="s">
         <v>495</v>
       </c>
-      <c r="F76" t="s">
-        <v>47</v>
-      </c>
-      <c r="G76" t="s">
-        <v>493</v>
-      </c>
       <c r="H76" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="I76" t="s">
-        <v>213</v>
+        <v>496</v>
       </c>
       <c r="J76" t="s">
         <v>21</v>
       </c>
       <c r="K76" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="L76" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="M76" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
     </row>
     <row r="77" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="B77">
         <v>1</v>
       </c>
       <c r="C77" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="D77" t="s">
+        <v>500</v>
+      </c>
+      <c r="E77" t="s">
+        <v>501</v>
+      </c>
+      <c r="F77" t="s">
+        <v>39</v>
+      </c>
+      <c r="G77" t="s">
         <v>499</v>
       </c>
-      <c r="E77" t="s">
-        <v>500</v>
-      </c>
-      <c r="F77" t="s">
-        <v>47</v>
-      </c>
-      <c r="G77" t="s">
-        <v>501</v>
-      </c>
       <c r="H77" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="I77" t="s">
+        <v>213</v>
+      </c>
+      <c r="J77" t="s">
+        <v>21</v>
+      </c>
+      <c r="K77" t="s">
         <v>502</v>
       </c>
-      <c r="J77" t="s">
-        <v>21</v>
-      </c>
-      <c r="K77" t="s">
-        <v>503</v>
-      </c>
       <c r="L77" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="M77" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
     </row>
     <row r="78" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
+        <v>503</v>
+      </c>
+      <c r="B78">
+        <v>1</v>
+      </c>
+      <c r="C78" t="s">
         <v>504</v>
       </c>
-      <c r="B78">
-        <v>2</v>
-      </c>
-      <c r="C78" t="s">
+      <c r="D78" t="s">
         <v>505</v>
       </c>
-      <c r="D78" t="s">
+      <c r="E78" t="s">
         <v>506</v>
       </c>
-      <c r="E78" t="s">
+      <c r="F78" t="s">
+        <v>39</v>
+      </c>
+      <c r="G78" t="s">
         <v>507</v>
       </c>
-      <c r="F78" t="s">
-        <v>47</v>
-      </c>
-      <c r="G78" t="s">
+      <c r="H78" t="s">
+        <v>504</v>
+      </c>
+      <c r="I78" t="s">
         <v>508</v>
       </c>
-      <c r="H78" t="s">
-        <v>505</v>
-      </c>
-      <c r="I78" t="s">
+      <c r="J78" t="s">
+        <v>21</v>
+      </c>
+      <c r="K78" t="s">
         <v>509</v>
       </c>
-      <c r="J78" t="s">
-        <v>21</v>
-      </c>
-      <c r="K78" t="s">
-        <v>510</v>
-      </c>
       <c r="L78" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="M78" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
     </row>
     <row r="79" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="B79">
         <v>1</v>
       </c>
       <c r="C79" t="s">
+        <v>511</v>
+      </c>
+      <c r="D79" t="s">
         <v>512</v>
       </c>
-      <c r="D79" t="s">
+      <c r="E79" t="s">
         <v>513</v>
       </c>
-      <c r="E79" t="s">
+      <c r="F79" t="s">
+        <v>39</v>
+      </c>
+      <c r="G79" t="s">
         <v>514</v>
       </c>
-      <c r="F79" t="s">
-        <v>47</v>
-      </c>
-      <c r="G79" t="s">
+      <c r="H79" t="s">
+        <v>511</v>
+      </c>
+      <c r="I79" t="s">
         <v>515</v>
       </c>
-      <c r="H79" t="s">
-        <v>512</v>
-      </c>
-      <c r="I79" t="s">
+      <c r="J79" t="s">
+        <v>21</v>
+      </c>
+      <c r="K79" t="s">
         <v>516</v>
       </c>
-      <c r="J79" t="s">
-        <v>21</v>
-      </c>
-      <c r="K79" t="s">
-        <v>517</v>
-      </c>
       <c r="L79" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="M79" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
     </row>
     <row r="80" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="B80">
         <v>1</v>
       </c>
       <c r="C80" t="s">
+        <v>518</v>
+      </c>
+      <c r="D80" t="s">
         <v>519</v>
-      </c>
-      <c r="D80" t="s">
-        <v>520</v>
       </c>
       <c r="E80" t="s">
         <v>437</v>
       </c>
       <c r="F80" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G80" t="s">
+        <v>520</v>
+      </c>
+      <c r="H80" t="s">
         <v>521</v>
-      </c>
-      <c r="H80" t="s">
-        <v>522</v>
       </c>
       <c r="I80" t="s">
         <v>440</v>
@@ -5257,39 +5254,39 @@
         <v>21</v>
       </c>
       <c r="K80" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="L80" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="M80" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="81" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="B81">
         <v>2</v>
       </c>
       <c r="C81" t="s">
+        <v>524</v>
+      </c>
+      <c r="D81" t="s">
         <v>525</v>
       </c>
-      <c r="D81" t="s">
+      <c r="E81" t="s">
         <v>526</v>
       </c>
-      <c r="E81" t="s">
+      <c r="F81" t="s">
+        <v>39</v>
+      </c>
+      <c r="G81" t="s">
         <v>527</v>
       </c>
-      <c r="F81" t="s">
-        <v>47</v>
-      </c>
-      <c r="G81" t="s">
+      <c r="H81" t="s">
         <v>528</v>
-      </c>
-      <c r="H81" t="s">
-        <v>529</v>
       </c>
       <c r="I81" t="s">
         <v>440</v>
@@ -5298,13 +5295,13 @@
         <v>21</v>
       </c>
       <c r="K81" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="L81" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="M81" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>